<commit_message>
fix: Python 2.7 sitecustomize 预加载 pyexpat 修复 xlrd 导出
</commit_message>
<xml_diff>
--- a/多语言翻译表.xlsx
+++ b/多语言翻译表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>::ID::</t>
   </si>
@@ -71,28 +71,16 @@
     <t>::JP::</t>
   </si>
   <si>
-    <t>Task_optimization15</t>
-  </si>
-  <si>
-    <t>({0}秒后自动关闭)</t>
-  </si>
-  <si>
-    <t>NEW_1v1_Des5</t>
-  </si>
-  <si>
-    <t>商店</t>
-  </si>
-  <si>
-    <t>D8_SSCM_Text18</t>
-  </si>
-  <si>
-    <t>挑战</t>
-  </si>
-  <si>
-    <t>D8_ShengWu_Text40</t>
-  </si>
-  <si>
-    <t>属性</t>
+    <t>D3_CorruptSecret_Text144</t>
+  </si>
+  <si>
+    <t>自动弹窗提醒队友求助</t>
+  </si>
+  <si>
+    <t>D3_CorruptSecret_Text145</t>
+  </si>
+  <si>
+    <t>联服已变更，腐败秘境的队伍发生变动，是否立刻前往查看？</t>
   </si>
 </sst>
 </file>
@@ -105,7 +93,14 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -258,7 +253,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,6 +262,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -452,12 +453,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -578,55 +594,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -641,79 +654,88 @@
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
@@ -999,7 +1021,7 @@
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="CCE8CF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1300,28 +1322,20 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">

</xml_diff>